<commit_message>
adds description of surface turbulence methods
</commit_message>
<xml_diff>
--- a/edi-mini-snorkel/data-raw/metadata/microhabitat_metadata.xlsx
+++ b/edi-mini-snorkel/data-raw/metadata/microhabitat_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashleyvizek/code/hrl/feather-river/edi-mini-snorkel/data-raw/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1D59D3-DA45-8C4B-9876-CC21563BFE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F77C39A-A68B-9146-B1D4-51F5EF555CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="66140" yWindow="1380" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -280,9 +280,6 @@
     <t>surface_turbulence</t>
   </si>
   <si>
-    <t>Surface turbulence measured within microhabitat plot</t>
-  </si>
-  <si>
     <t>centimeter</t>
   </si>
   <si>
@@ -294,6 +291,9 @@
   </si>
   <si>
     <t>Indicates is fish is hatchery origin is wild. This was only recorded for steelhead.</t>
+  </si>
+  <si>
+    <t>Surface turbulence refers to the rapid and multi-directional movement of water at the air-water interface, often appearing as choppy water, riffles, or small breaking waves. It was measured by finding the percentage of each 1x1 m grid that is covered by surface turbulence.  The level of turbulence is not described, only if its present or not and how much of the grid had some level of turbulence (e.g. minor rippling of the surface was counted the same as “white water”).</t>
   </si>
 </sst>
 </file>
@@ -936,7 +936,7 @@
         <v>59</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
@@ -971,10 +971,10 @@
     </row>
     <row r="9" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>13</v>
@@ -1075,7 +1075,7 @@
         <v>15</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>17</v>
@@ -1123,7 +1123,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>17</v>
@@ -1252,7 +1252,7 @@
         <v>83</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>15</v>

</xml_diff>